<commit_message>
separate test script and data
</commit_message>
<xml_diff>
--- a/backend/ArchClub_Test_Report.xlsx
+++ b/backend/ArchClub_Test_Report.xlsx
@@ -1,37 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27932"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\DataDrivenTesting\backend\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13D845C3-DE4B-4889-8F41-7909693462DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -62,6 +40,9 @@
     <t>Tested By:</t>
   </si>
   <si>
+    <t>Sinh viên thực hiện</t>
+  </si>
+  <si>
     <t>Function Name</t>
   </si>
   <si>
@@ -90,16 +71,13 @@
   </si>
   <si>
     <t>GRAND TOTAL</t>
-  </si>
-  <si>
-    <t>Nguyễn Thành Thái</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -187,42 +165,25 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="110"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="10"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
+  <c:style val="10"/>
   <c:chart>
     <c:title>
       <c:tx>
@@ -240,9 +201,8 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:overlay val="0"/>
+      <c:layout/>
     </c:title>
-    <c:autoTitleDeleted val="0"/>
     <c:plotArea>
       <c:layout/>
       <c:pieChart>
@@ -255,50 +215,23 @@
           </c:tx>
           <c:dPt>
             <c:idx val="0"/>
-            <c:bubble3D val="0"/>
             <c:spPr>
               <a:solidFill>
                 <a:srgbClr val="1D70B8"/>
               </a:solidFill>
             </c:spPr>
-            <c:extLst>
-              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000000-C762-44AD-AE29-284947C98EEB}"/>
-              </c:ext>
-            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
-            <c:bubble3D val="0"/>
             <c:spPr>
               <a:solidFill>
                 <a:srgbClr val="D4351C"/>
               </a:solidFill>
             </c:spPr>
-            <c:extLst>
-              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000001-C762-44AD-AE29-284947C98EEB}"/>
-              </c:ext>
-            </c:extLst>
           </c:dPt>
           <c:dLbls>
-            <c:spPr>
-              <a:noFill/>
-              <a:ln>
-                <a:noFill/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-            <c:showLegendKey val="0"/>
             <c:showVal val="1"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
             <c:showPercent val="1"/>
-            <c:showBubbleSize val="0"/>
-            <c:showLeaderLines val="0"/>
-            <c:extLst>
-              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
-            </c:extLst>
           </c:dLbls>
           <c:cat>
             <c:strRef>
@@ -329,27 +262,13 @@
               </c:numCache>
             </c:numRef>
           </c:val>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-C762-44AD-AE29-284947C98EEB}"/>
-            </c:ext>
-          </c:extLst>
         </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-          <c:showLeaderLines val="0"/>
-        </c:dLbls>
         <c:firstSliceAng val="0"/>
       </c:pieChart>
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
-      <c:overlay val="0"/>
+      <c:layout/>
       <c:txPr>
         <a:bodyPr/>
         <a:lstStyle/>
@@ -362,8 +281,6 @@
       </c:txPr>
     </c:legend>
     <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:printSettings>
     <c:headerFooter/>
@@ -390,13 +307,7 @@
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -415,9 +326,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -455,7 +366,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -489,7 +400,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -524,10 +434,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -700,147 +609,145 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.7109375" customWidth="1"/>
-    <col min="2" max="2" width="21" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:4">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:4">
+      <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="3">
+        <v>12</v>
+      </c>
+      <c r="C7" s="3">
+        <v>3</v>
+      </c>
+      <c r="D7" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="3">
+        <v>14</v>
+      </c>
+      <c r="C8" s="3">
+        <v>2</v>
+      </c>
+      <c r="D8" s="3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="3">
+        <v>9</v>
+      </c>
+      <c r="C9" s="3">
+        <v>3</v>
+      </c>
+      <c r="D9" s="3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="3">
+        <v>10</v>
+      </c>
+      <c r="C10" s="3">
+        <v>0</v>
+      </c>
+      <c r="D10" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="3">
+        <v>4</v>
+      </c>
+      <c r="C11" s="3">
+        <v>0</v>
+      </c>
+      <c r="D11" s="3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" s="2" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+      <c r="B12" s="2">
+        <v>49</v>
+      </c>
+      <c r="C12" s="2">
         <v>8</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="2">
-        <v>12</v>
-      </c>
-      <c r="C7" s="2">
-        <v>3</v>
-      </c>
-      <c r="D7" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" s="2">
-        <v>14</v>
-      </c>
-      <c r="C8" s="2">
-        <v>2</v>
-      </c>
-      <c r="D8" s="2">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="2">
-        <v>9</v>
-      </c>
-      <c r="C9" s="2">
-        <v>3</v>
-      </c>
-      <c r="D9" s="2">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" s="2">
-        <v>10</v>
-      </c>
-      <c r="C10" s="2">
-        <v>0</v>
-      </c>
-      <c r="D10" s="2">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" s="2">
-        <v>4</v>
-      </c>
-      <c r="C11" s="2">
-        <v>0</v>
-      </c>
-      <c r="D11" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B12" s="1">
-        <v>49</v>
-      </c>
-      <c r="C12" s="1">
-        <v>8</v>
-      </c>
-      <c r="D12" s="1">
+      <c r="D12" s="2">
         <v>57</v>
       </c>
     </row>

</xml_diff>